<commit_message>
Add standalone vulnerability categorization and update ablation workflow
</commit_message>
<xml_diff>
--- a/data/sample/midhili/Cyclone_Midhili_Observed_Damage_Data.xlsx
+++ b/data/sample/midhili/Cyclone_Midhili_Observed_Damage_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ibrahim\IBF-Analysis\data\sample\midhili\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA82EB68-0840-447B-A1AE-378FBFE08FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E8E504-5DA7-4031-87E0-E64A620E6110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="House" sheetId="2" r:id="rId1"/>

</xml_diff>